<commit_message>
Impegni degli studenti e attesa dopo il mattino
Nuovo foglio "Impegni studenti": una griglia come quella dei docenti ma al
contrario, dove la X segna l'ora in cui il ragazzo NON può esserci. È un
vincolo rigido e si somma ai giorni vietati del foglio Studenti. Un pulsante
copia l'elenco dei nomi dal foglio Studenti. I file creati prima non hanno il
foglio: viene aggiunto vuoto all'apertura.

Analizzando l'orario prodotto è emerso che il programma contava i buchi fra le
lezioni del pomeriggio ma non l'attesa fra la fine del mattino e la prima
lezione, che per chi resta a scuola è tempo perso uguale: da qui le lezioni
isolate a metà pomeriggio. Ora quell'attesa ha un costo, più alto per chi
abita lontano. Sui dati veri le ore di attesa passano da 128 a 80, i pomeriggi
che cominciano alle 16:30 da 19 a 5 e i ragazzi che vengono un solo pomeriggio
da 50 a 65, sempre senza buchi.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/esempio/orario_2026-27.xlsx
+++ b/esempio/orario_2026-27.xlsx
@@ -9,10 +9,11 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Istruzioni" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Studenti" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Docenti" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppi LMC" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LMI" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parametri" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Impegni studenti" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Docenti" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppi LMC" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LMI" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parametri" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -438,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A40"/>
+  <dimension ref="A1:A45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="115" customWidth="1" min="1" max="1"/>
@@ -630,67 +631,98 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>FOGLIO 'LMI' – laboratori di musica d'insieme (2 ore, orario del MATTINO). Un rigo per laboratorio.</t>
+          <t>FOGLIO 'Impegni studenti' – le ore in cui un ragazzo NON può venire (sport, catechismo, altro).</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Il programma NON li calcola: li ricopia così come sono in una pagina dell'orario.</t>
+          <t xml:space="preserve">  ATTENZIONE: qui è al contrario del foglio Docenti. La X segna l'ora in cui il ragazzo NON c'è.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Studenti: 'Cognome Nome' separati da virgola. Anche qui il nome viene aggiunto da solo quando non ci sono omonimi.</t>
+          <t xml:space="preserve">  Chi non ha impegni si lascia con la riga vuota. Nel programma il pulsante 'Compila dagli studenti'</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" t="inlineStr"/>
+      <c r="A33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ricopia l'elenco dei nomi dal foglio Studenti.</t>
+        </is>
+      </c>
     </row>
     <row r="34">
-      <c r="A34" s="2" t="inlineStr">
-        <is>
-          <t>FOGLIO 'Parametri' – poche regole generali (max rientri, tempo di calcolo). Di norma non serve toccarlo.</t>
-        </is>
-      </c>
+      <c r="A34" t="inlineStr"/>
     </row>
     <row r="35">
-      <c r="A35" t="inlineStr"/>
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>FOGLIO 'LMI' – laboratori di musica d'insieme (2 ore, orario del MATTINO). Un rigo per laboratorio.</t>
+        </is>
+      </c>
     </row>
     <row r="36">
-      <c r="A36" s="2" t="inlineStr">
-        <is>
-          <t>REGOLE FISSE (non modificabili da qui):</t>
+      <c r="A36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Il programma NON li calcola: li ricopia così come sono in una pagina dell'orario.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
+          <t xml:space="preserve">  Studenti: 'Cognome Nome' separati da virgola. Anche qui il nome viene aggiunto da solo quando non ci sono omonimi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>FOGLIO 'Parametri' – poche regole generali (max rientri, tempo di calcolo). Di norma non serve toccarlo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>REGOLE FISSE (non modificabili da qui):</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
           <t xml:space="preserve">  Classi 1 e 2: 2 ore 1° strumento + 1 ora 2° strumento.</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
+    <row r="43">
+      <c r="A43" t="inlineStr">
         <is>
           <t xml:space="preserve">  Classi 3 e 4: 1 ora 1° strumento + 1 ora 2° strumento + 1 ora musica da camera.</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
+    <row r="44">
+      <c r="A44" t="inlineStr">
         <is>
           <t xml:space="preserve">  Classe 5:     2 ore 1° strumento + 1 ora musica da camera.</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
+    <row r="45">
+      <c r="A45" t="inlineStr">
         <is>
           <t xml:space="preserve">  Fasce: 13:30-14:30, 14:30-15:30, 15:30-16:30, 16:30-17:30, da lunedì a venerdì.</t>
         </is>
@@ -2744,6 +2776,1321 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:X31"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="7" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="6.5" customWidth="1" min="4" max="4"/>
+    <col width="6.5" customWidth="1" min="5" max="5"/>
+    <col width="6.5" customWidth="1" min="6" max="6"/>
+    <col width="6.5" customWidth="1" min="7" max="7"/>
+    <col width="6.5" customWidth="1" min="8" max="8"/>
+    <col width="6.5" customWidth="1" min="9" max="9"/>
+    <col width="6.5" customWidth="1" min="10" max="10"/>
+    <col width="6.5" customWidth="1" min="11" max="11"/>
+    <col width="6.5" customWidth="1" min="12" max="12"/>
+    <col width="6.5" customWidth="1" min="13" max="13"/>
+    <col width="6.5" customWidth="1" min="14" max="14"/>
+    <col width="6.5" customWidth="1" min="15" max="15"/>
+    <col width="6.5" customWidth="1" min="16" max="16"/>
+    <col width="6.5" customWidth="1" min="17" max="17"/>
+    <col width="6.5" customWidth="1" min="18" max="18"/>
+    <col width="6.5" customWidth="1" min="19" max="19"/>
+    <col width="6.5" customWidth="1" min="20" max="20"/>
+    <col width="6.5" customWidth="1" min="21" max="21"/>
+    <col width="6.5" customWidth="1" min="22" max="22"/>
+    <col width="6.5" customWidth="1" min="23" max="23"/>
+    <col width="30" customWidth="1" min="24" max="24"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="60" customHeight="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Classe</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>Cognome</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>Nome</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>Lun 13:30</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>Lun 14:30</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>Lun 15:30</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>Lun 16:30</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>Mar 13:30</t>
+        </is>
+      </c>
+      <c r="I1" s="4" t="inlineStr">
+        <is>
+          <t>Mar 14:30</t>
+        </is>
+      </c>
+      <c r="J1" s="4" t="inlineStr">
+        <is>
+          <t>Mar 15:30</t>
+        </is>
+      </c>
+      <c r="K1" s="4" t="inlineStr">
+        <is>
+          <t>Mar 16:30</t>
+        </is>
+      </c>
+      <c r="L1" s="4" t="inlineStr">
+        <is>
+          <t>Mer 13:30</t>
+        </is>
+      </c>
+      <c r="M1" s="4" t="inlineStr">
+        <is>
+          <t>Mer 14:30</t>
+        </is>
+      </c>
+      <c r="N1" s="4" t="inlineStr">
+        <is>
+          <t>Mer 15:30</t>
+        </is>
+      </c>
+      <c r="O1" s="4" t="inlineStr">
+        <is>
+          <t>Mer 16:30</t>
+        </is>
+      </c>
+      <c r="P1" s="4" t="inlineStr">
+        <is>
+          <t>Gio 13:30</t>
+        </is>
+      </c>
+      <c r="Q1" s="4" t="inlineStr">
+        <is>
+          <t>Gio 14:30</t>
+        </is>
+      </c>
+      <c r="R1" s="4" t="inlineStr">
+        <is>
+          <t>Gio 15:30</t>
+        </is>
+      </c>
+      <c r="S1" s="4" t="inlineStr">
+        <is>
+          <t>Gio 16:30</t>
+        </is>
+      </c>
+      <c r="T1" s="4" t="inlineStr">
+        <is>
+          <t>Ven 13:30</t>
+        </is>
+      </c>
+      <c r="U1" s="4" t="inlineStr">
+        <is>
+          <t>Ven 14:30</t>
+        </is>
+      </c>
+      <c r="V1" s="4" t="inlineStr">
+        <is>
+          <t>Ven 15:30</t>
+        </is>
+      </c>
+      <c r="W1" s="4" t="inlineStr">
+        <is>
+          <t>Ven 16:30</t>
+        </is>
+      </c>
+      <c r="X1" s="3" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>AMATO</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>GIULIA</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr"/>
+      <c r="Q2" t="inlineStr"/>
+      <c r="R2" t="inlineStr"/>
+      <c r="S2" t="inlineStr"/>
+      <c r="T2" t="inlineStr"/>
+      <c r="U2" t="inlineStr"/>
+      <c r="V2" t="inlineStr"/>
+      <c r="W2" t="inlineStr"/>
+      <c r="X2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>BRUNI</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>MATTEO</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr"/>
+      <c r="Q3" t="inlineStr"/>
+      <c r="R3" t="inlineStr"/>
+      <c r="S3" t="inlineStr"/>
+      <c r="T3" t="inlineStr"/>
+      <c r="U3" t="inlineStr"/>
+      <c r="V3" t="inlineStr"/>
+      <c r="W3" t="inlineStr"/>
+      <c r="X3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>CARRARA</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>SOFIA</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr"/>
+      <c r="Q4" t="inlineStr"/>
+      <c r="R4" t="inlineStr"/>
+      <c r="S4" t="inlineStr"/>
+      <c r="T4" t="inlineStr"/>
+      <c r="U4" t="inlineStr"/>
+      <c r="V4" t="inlineStr"/>
+      <c r="W4" t="inlineStr"/>
+      <c r="X4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>DONATI</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>LORENZO</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" t="inlineStr"/>
+      <c r="Q5" t="inlineStr"/>
+      <c r="R5" t="inlineStr"/>
+      <c r="S5" t="inlineStr"/>
+      <c r="T5" t="inlineStr"/>
+      <c r="U5" t="inlineStr"/>
+      <c r="V5" t="inlineStr"/>
+      <c r="W5" t="inlineStr"/>
+      <c r="X5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ESPOSITO</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>CHIARA</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr"/>
+      <c r="P6" t="inlineStr"/>
+      <c r="Q6" t="inlineStr"/>
+      <c r="R6" t="inlineStr"/>
+      <c r="S6" t="inlineStr"/>
+      <c r="T6" t="inlineStr"/>
+      <c r="U6" t="inlineStr"/>
+      <c r="V6" t="inlineStr"/>
+      <c r="W6" t="inlineStr"/>
+      <c r="X6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>1</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>FANTI</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>TOMMASO</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr"/>
+      <c r="P7" t="inlineStr"/>
+      <c r="Q7" t="inlineStr"/>
+      <c r="R7" t="inlineStr"/>
+      <c r="S7" t="inlineStr"/>
+      <c r="T7" t="inlineStr"/>
+      <c r="U7" t="inlineStr"/>
+      <c r="V7" t="inlineStr"/>
+      <c r="W7" t="inlineStr"/>
+      <c r="X7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>1</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>GRASSI</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>ALICE</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" t="inlineStr"/>
+      <c r="O8" t="inlineStr"/>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr"/>
+      <c r="R8" t="inlineStr"/>
+      <c r="S8" t="inlineStr"/>
+      <c r="T8" t="inlineStr"/>
+      <c r="U8" t="inlineStr"/>
+      <c r="V8" t="inlineStr"/>
+      <c r="W8" t="inlineStr"/>
+      <c r="X8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>1</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>LUPI</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>FEDERICO</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr"/>
+      <c r="N9" t="inlineStr"/>
+      <c r="O9" t="inlineStr"/>
+      <c r="P9" t="inlineStr"/>
+      <c r="Q9" t="inlineStr"/>
+      <c r="R9" t="inlineStr"/>
+      <c r="S9" t="inlineStr"/>
+      <c r="T9" t="inlineStr"/>
+      <c r="U9" t="inlineStr"/>
+      <c r="V9" t="inlineStr"/>
+      <c r="W9" t="inlineStr"/>
+      <c r="X9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>2</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>MARCHI</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>EMMA</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr"/>
+      <c r="N10" t="inlineStr"/>
+      <c r="O10" t="inlineStr"/>
+      <c r="P10" t="inlineStr"/>
+      <c r="Q10" t="inlineStr"/>
+      <c r="R10" t="inlineStr"/>
+      <c r="S10" t="inlineStr"/>
+      <c r="T10" t="inlineStr"/>
+      <c r="U10" t="inlineStr"/>
+      <c r="V10" t="inlineStr"/>
+      <c r="W10" t="inlineStr"/>
+      <c r="X10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>2</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>NARDI</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>GABRIELE</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr"/>
+      <c r="N11" t="inlineStr"/>
+      <c r="O11" t="inlineStr"/>
+      <c r="P11" t="inlineStr"/>
+      <c r="Q11" t="inlineStr"/>
+      <c r="R11" t="inlineStr"/>
+      <c r="S11" t="inlineStr"/>
+      <c r="T11" t="inlineStr"/>
+      <c r="U11" t="inlineStr"/>
+      <c r="V11" t="inlineStr"/>
+      <c r="W11" t="inlineStr"/>
+      <c r="X11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>2</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>ORLANDI</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>VIOLA</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="inlineStr"/>
+      <c r="N12" t="inlineStr"/>
+      <c r="O12" t="inlineStr"/>
+      <c r="P12" t="inlineStr"/>
+      <c r="Q12" t="inlineStr"/>
+      <c r="R12" t="inlineStr"/>
+      <c r="S12" t="inlineStr"/>
+      <c r="T12" t="inlineStr"/>
+      <c r="U12" t="inlineStr"/>
+      <c r="V12" t="inlineStr"/>
+      <c r="W12" t="inlineStr"/>
+      <c r="X12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>2</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>PIERI</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>LEONARDO</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="inlineStr"/>
+      <c r="N13" t="inlineStr"/>
+      <c r="O13" t="inlineStr"/>
+      <c r="P13" t="inlineStr"/>
+      <c r="Q13" t="inlineStr"/>
+      <c r="R13" t="inlineStr"/>
+      <c r="S13" t="inlineStr"/>
+      <c r="T13" t="inlineStr"/>
+      <c r="U13" t="inlineStr"/>
+      <c r="V13" t="inlineStr"/>
+      <c r="W13" t="inlineStr"/>
+      <c r="X13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>2</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>RENZI</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>MARTINA</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr"/>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr"/>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr"/>
+      <c r="L14" t="inlineStr"/>
+      <c r="M14" t="inlineStr"/>
+      <c r="N14" t="inlineStr"/>
+      <c r="O14" t="inlineStr"/>
+      <c r="P14" t="inlineStr"/>
+      <c r="Q14" t="inlineStr"/>
+      <c r="R14" t="inlineStr"/>
+      <c r="S14" t="inlineStr"/>
+      <c r="T14" t="inlineStr"/>
+      <c r="U14" t="inlineStr"/>
+      <c r="V14" t="inlineStr"/>
+      <c r="W14" t="inlineStr"/>
+      <c r="X14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>2</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>SARTI</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>DIEGO</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr"/>
+      <c r="L15" t="inlineStr"/>
+      <c r="M15" t="inlineStr"/>
+      <c r="N15" t="inlineStr"/>
+      <c r="O15" t="inlineStr"/>
+      <c r="P15" t="inlineStr"/>
+      <c r="Q15" t="inlineStr"/>
+      <c r="R15" t="inlineStr"/>
+      <c r="S15" t="inlineStr"/>
+      <c r="T15" t="inlineStr"/>
+      <c r="U15" t="inlineStr"/>
+      <c r="V15" t="inlineStr"/>
+      <c r="W15" t="inlineStr"/>
+      <c r="X15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>3</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>BANDINI</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>FILIPPO</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr"/>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr"/>
+      <c r="L16" t="inlineStr"/>
+      <c r="M16" t="inlineStr"/>
+      <c r="N16" t="inlineStr"/>
+      <c r="O16" t="inlineStr"/>
+      <c r="P16" t="inlineStr"/>
+      <c r="Q16" t="inlineStr"/>
+      <c r="R16" t="inlineStr"/>
+      <c r="S16" t="inlineStr"/>
+      <c r="T16" t="inlineStr"/>
+      <c r="U16" t="inlineStr"/>
+      <c r="V16" t="inlineStr"/>
+      <c r="W16" t="inlineStr"/>
+      <c r="X16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>3</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>CECCONI</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>GAIA</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr"/>
+      <c r="L17" t="inlineStr"/>
+      <c r="M17" t="inlineStr"/>
+      <c r="N17" t="inlineStr"/>
+      <c r="O17" t="inlineStr"/>
+      <c r="P17" t="inlineStr"/>
+      <c r="Q17" t="inlineStr"/>
+      <c r="R17" t="inlineStr"/>
+      <c r="S17" t="inlineStr"/>
+      <c r="T17" t="inlineStr"/>
+      <c r="U17" t="inlineStr"/>
+      <c r="V17" t="inlineStr"/>
+      <c r="W17" t="inlineStr"/>
+      <c r="X17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>3</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>DINI</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>RICCARDO</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr"/>
+      <c r="L18" t="inlineStr"/>
+      <c r="M18" t="inlineStr"/>
+      <c r="N18" t="inlineStr"/>
+      <c r="O18" t="inlineStr"/>
+      <c r="P18" t="inlineStr"/>
+      <c r="Q18" t="inlineStr"/>
+      <c r="R18" t="inlineStr"/>
+      <c r="S18" t="inlineStr"/>
+      <c r="T18" t="inlineStr"/>
+      <c r="U18" t="inlineStr"/>
+      <c r="V18" t="inlineStr"/>
+      <c r="W18" t="inlineStr"/>
+      <c r="X18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>3</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>TOSI</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>BEATRICE</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr"/>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr"/>
+      <c r="J19" t="inlineStr"/>
+      <c r="K19" t="inlineStr"/>
+      <c r="L19" t="inlineStr"/>
+      <c r="M19" t="inlineStr"/>
+      <c r="N19" t="inlineStr"/>
+      <c r="O19" t="inlineStr"/>
+      <c r="P19" t="inlineStr"/>
+      <c r="Q19" t="inlineStr"/>
+      <c r="R19" t="inlineStr"/>
+      <c r="S19" t="inlineStr"/>
+      <c r="T19" t="inlineStr"/>
+      <c r="U19" t="inlineStr"/>
+      <c r="V19" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="W19" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="X19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>3</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>VESTRI</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>SAMUELE</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="inlineStr"/>
+      <c r="K20" t="inlineStr"/>
+      <c r="L20" t="inlineStr"/>
+      <c r="M20" t="inlineStr"/>
+      <c r="N20" t="inlineStr"/>
+      <c r="O20" t="inlineStr"/>
+      <c r="P20" t="inlineStr"/>
+      <c r="Q20" t="inlineStr"/>
+      <c r="R20" t="inlineStr"/>
+      <c r="S20" t="inlineStr"/>
+      <c r="T20" t="inlineStr"/>
+      <c r="U20" t="inlineStr"/>
+      <c r="V20" t="inlineStr"/>
+      <c r="W20" t="inlineStr"/>
+      <c r="X20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>3</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>ZACCARIA</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>NOEMI</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="inlineStr"/>
+      <c r="K21" t="inlineStr"/>
+      <c r="L21" t="inlineStr"/>
+      <c r="M21" t="inlineStr"/>
+      <c r="N21" t="inlineStr"/>
+      <c r="O21" t="inlineStr"/>
+      <c r="P21" t="inlineStr"/>
+      <c r="Q21" t="inlineStr"/>
+      <c r="R21" t="inlineStr"/>
+      <c r="S21" t="inlineStr"/>
+      <c r="T21" t="inlineStr"/>
+      <c r="U21" t="inlineStr"/>
+      <c r="V21" t="inlineStr"/>
+      <c r="W21" t="inlineStr"/>
+      <c r="X21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>4</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>FIORI</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>ELISA</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr"/>
+      <c r="E22" t="inlineStr"/>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr"/>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr"/>
+      <c r="J22" t="inlineStr"/>
+      <c r="K22" t="inlineStr"/>
+      <c r="L22" t="inlineStr"/>
+      <c r="M22" t="inlineStr"/>
+      <c r="N22" t="inlineStr"/>
+      <c r="O22" t="inlineStr"/>
+      <c r="P22" t="inlineStr"/>
+      <c r="Q22" t="inlineStr"/>
+      <c r="R22" t="inlineStr"/>
+      <c r="S22" t="inlineStr"/>
+      <c r="T22" t="inlineStr"/>
+      <c r="U22" t="inlineStr"/>
+      <c r="V22" t="inlineStr"/>
+      <c r="W22" t="inlineStr"/>
+      <c r="X22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>4</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>GARGINI</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>NICOLA</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr"/>
+      <c r="E23" t="inlineStr"/>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr"/>
+      <c r="J23" t="inlineStr"/>
+      <c r="K23" t="inlineStr"/>
+      <c r="L23" t="inlineStr"/>
+      <c r="M23" t="inlineStr"/>
+      <c r="N23" t="inlineStr"/>
+      <c r="O23" t="inlineStr"/>
+      <c r="P23" t="inlineStr"/>
+      <c r="Q23" t="inlineStr"/>
+      <c r="R23" t="inlineStr"/>
+      <c r="S23" t="inlineStr"/>
+      <c r="T23" t="inlineStr"/>
+      <c r="U23" t="inlineStr"/>
+      <c r="V23" t="inlineStr"/>
+      <c r="W23" t="inlineStr"/>
+      <c r="X23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>4</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>LAZZERI</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>ARIANNA</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr"/>
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr"/>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr"/>
+      <c r="J24" t="inlineStr"/>
+      <c r="K24" t="inlineStr"/>
+      <c r="L24" t="inlineStr"/>
+      <c r="M24" t="inlineStr"/>
+      <c r="N24" t="inlineStr"/>
+      <c r="O24" t="inlineStr"/>
+      <c r="P24" t="inlineStr"/>
+      <c r="Q24" t="inlineStr"/>
+      <c r="R24" t="inlineStr"/>
+      <c r="S24" t="inlineStr"/>
+      <c r="T24" t="inlineStr"/>
+      <c r="U24" t="inlineStr"/>
+      <c r="V24" t="inlineStr"/>
+      <c r="W24" t="inlineStr"/>
+      <c r="X24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>4</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>MERLI</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>ANDREA</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr"/>
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="inlineStr"/>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr"/>
+      <c r="J25" t="inlineStr"/>
+      <c r="K25" t="inlineStr"/>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr"/>
+      <c r="N25" t="inlineStr"/>
+      <c r="O25" t="inlineStr"/>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="Q25" t="inlineStr"/>
+      <c r="R25" t="inlineStr"/>
+      <c r="S25" t="inlineStr"/>
+      <c r="T25" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="U25" t="inlineStr"/>
+      <c r="V25" t="inlineStr"/>
+      <c r="W25" t="inlineStr"/>
+      <c r="X25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>4</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>NESTI</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>GIORGIA</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr"/>
+      <c r="E26" t="inlineStr"/>
+      <c r="F26" t="inlineStr"/>
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="inlineStr"/>
+      <c r="J26" t="inlineStr"/>
+      <c r="K26" t="inlineStr"/>
+      <c r="L26" t="inlineStr"/>
+      <c r="M26" t="inlineStr"/>
+      <c r="N26" t="inlineStr"/>
+      <c r="O26" t="inlineStr"/>
+      <c r="P26" t="inlineStr"/>
+      <c r="Q26" t="inlineStr"/>
+      <c r="R26" t="inlineStr"/>
+      <c r="S26" t="inlineStr"/>
+      <c r="T26" t="inlineStr"/>
+      <c r="U26" t="inlineStr"/>
+      <c r="V26" t="inlineStr"/>
+      <c r="W26" t="inlineStr"/>
+      <c r="X26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>5</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>PAGNI</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>DAVIDE</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr"/>
+      <c r="E27" t="inlineStr"/>
+      <c r="F27" t="inlineStr"/>
+      <c r="G27" t="inlineStr"/>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="inlineStr"/>
+      <c r="J27" t="inlineStr"/>
+      <c r="K27" t="inlineStr"/>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="P27" t="inlineStr"/>
+      <c r="Q27" t="inlineStr"/>
+      <c r="R27" t="inlineStr"/>
+      <c r="S27" t="inlineStr"/>
+      <c r="T27" t="inlineStr"/>
+      <c r="U27" t="inlineStr"/>
+      <c r="V27" t="inlineStr"/>
+      <c r="W27" t="inlineStr"/>
+      <c r="X27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>5</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>QUERCI</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>SARA</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr"/>
+      <c r="E28" t="inlineStr"/>
+      <c r="F28" t="inlineStr"/>
+      <c r="G28" t="inlineStr"/>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr"/>
+      <c r="J28" t="inlineStr"/>
+      <c r="K28" t="inlineStr"/>
+      <c r="L28" t="inlineStr"/>
+      <c r="M28" t="inlineStr"/>
+      <c r="N28" t="inlineStr"/>
+      <c r="O28" t="inlineStr"/>
+      <c r="P28" t="inlineStr"/>
+      <c r="Q28" t="inlineStr"/>
+      <c r="R28" t="inlineStr"/>
+      <c r="S28" t="inlineStr"/>
+      <c r="T28" t="inlineStr"/>
+      <c r="U28" t="inlineStr"/>
+      <c r="V28" t="inlineStr"/>
+      <c r="W28" t="inlineStr"/>
+      <c r="X28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>5</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>SALVI</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>MARCO</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr"/>
+      <c r="E29" t="inlineStr"/>
+      <c r="F29" t="inlineStr"/>
+      <c r="G29" t="inlineStr"/>
+      <c r="H29" t="inlineStr"/>
+      <c r="I29" t="inlineStr"/>
+      <c r="J29" t="inlineStr"/>
+      <c r="K29" t="inlineStr"/>
+      <c r="L29" t="inlineStr"/>
+      <c r="M29" t="inlineStr"/>
+      <c r="N29" t="inlineStr"/>
+      <c r="O29" t="inlineStr"/>
+      <c r="P29" t="inlineStr"/>
+      <c r="Q29" t="inlineStr"/>
+      <c r="R29" t="inlineStr"/>
+      <c r="S29" t="inlineStr"/>
+      <c r="T29" t="inlineStr"/>
+      <c r="U29" t="inlineStr"/>
+      <c r="V29" t="inlineStr"/>
+      <c r="W29" t="inlineStr"/>
+      <c r="X29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>5</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>TURCHI</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>LUCIA</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr"/>
+      <c r="E30" t="inlineStr"/>
+      <c r="F30" t="inlineStr"/>
+      <c r="G30" t="inlineStr"/>
+      <c r="H30" t="inlineStr"/>
+      <c r="I30" t="inlineStr"/>
+      <c r="J30" t="inlineStr"/>
+      <c r="K30" t="inlineStr"/>
+      <c r="L30" t="inlineStr"/>
+      <c r="M30" t="inlineStr"/>
+      <c r="N30" t="inlineStr"/>
+      <c r="O30" t="inlineStr"/>
+      <c r="P30" t="inlineStr"/>
+      <c r="Q30" t="inlineStr"/>
+      <c r="R30" t="inlineStr"/>
+      <c r="S30" t="inlineStr"/>
+      <c r="T30" t="inlineStr"/>
+      <c r="U30" t="inlineStr"/>
+      <c r="V30" t="inlineStr"/>
+      <c r="W30" t="inlineStr"/>
+      <c r="X30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>5</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>VENTURI</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>PIETRO</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr"/>
+      <c r="E31" t="inlineStr"/>
+      <c r="F31" t="inlineStr"/>
+      <c r="G31" t="inlineStr"/>
+      <c r="H31" t="inlineStr"/>
+      <c r="I31" t="inlineStr"/>
+      <c r="J31" t="inlineStr"/>
+      <c r="K31" t="inlineStr"/>
+      <c r="L31" t="inlineStr"/>
+      <c r="M31" t="inlineStr"/>
+      <c r="N31" t="inlineStr"/>
+      <c r="O31" t="inlineStr"/>
+      <c r="P31" t="inlineStr"/>
+      <c r="Q31" t="inlineStr"/>
+      <c r="R31" t="inlineStr"/>
+      <c r="S31" t="inlineStr"/>
+      <c r="T31" t="inlineStr"/>
+      <c r="U31" t="inlineStr"/>
+      <c r="V31" t="inlineStr"/>
+      <c r="W31" t="inlineStr"/>
+      <c r="X31" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="D2:W231" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"X"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3835,7 +5182,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4069,7 +5416,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4200,7 +5547,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Colonna «1° strumento attaccato»: SI, NO oppure lasciare decidere
Sostituisce «Ore consecutive» e ha tre stati. SI: le 2 ore di 1°
strumento una di seguito all'altra, come prima. NO: in due giorni
diversi, quindi mai attaccate — vincolo nuovo nel modello, una sola
delle due ore per giorno. Vuoto: decide il programma.

Vale per le classi 1ª, 2ª e 5ª, le uniche con 2 ore; altrove è un
avviso. I controlli fermano prima le richieste impossibili: per il SI
servono due ore consecutive libere dello stesso docente, per il NO
almeno due giorni.

Aprendo un file di una versione precedente la colonna viene rinominata
mantenendo i SI già scritti, e la lettura accetta comunque il vecchio
titolo. Nel file di esempio due ragazzi di 2ª hanno adesso il NO.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/esempio/orario_2026-27.xlsx
+++ b/esempio/orario_2026-27.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A49"/>
+  <dimension ref="A1:A55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="115" customWidth="1" min="1" max="1"/>
@@ -497,257 +497,299 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Ore consecutive = SI se le 2 ore di 1° strumento devono essere una di seguito all'altra (solo classi 1, 2, 5).</t>
+          <t xml:space="preserve">  1° strumento attaccato (solo classi 1, 2, 5, che hanno 2 ore): SI = le due ore una di seguito all'altra,</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Giorno unico = SI se il ragazzo deve rientrare un solo giorno a settimana.</t>
+          <t xml:space="preserve">  NO = in due giorni diversi, casella vuota = decide il programma.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Giorni NON disponibili: es. 'Mar, Gio' se il ragazzo non può venire quei pomeriggi. Vuoto = tutti i giorni possibili.</t>
+          <t xml:space="preserve">  Giorno unico = SI se il ragazzo deve rientrare un solo giorno a settimana.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Comune, Indirizzo, Civico: per calcolare i tempi di ritorno a casa con i mezzi (menu Orario → Aggiorna trasporti).</t>
+          <t xml:space="preserve">  Giorni NON disponibili: es. 'Mar, Gio' se il ragazzo non può venire quei pomeriggi. Vuoto = tutti i giorni possibili.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
+          <t xml:space="preserve">  Comune, Indirizzo, Civico: per calcolare i tempi di ritorno a casa con i mezzi (menu Orario → Aggiorna trasporti).</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
           <t xml:space="preserve">  KM: distanza casa-scuola, usata quando mancano i dati dei mezzi. Senza né KM né mezzi si è trattati come vicini.</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="inlineStr"/>
-    </row>
     <row r="15">
-      <c r="A15" s="2" t="inlineStr">
+      <c r="A15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
         <is>
           <t>FOGLIO 'Docenti' – un rigo per docente, con la disponibilità oraria.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Nel programma il pulsante 'Compila dagli studenti' aggiunge da solo i docenti che compaiono nel foglio</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Studenti e nei gruppi, con i loro strumenti: restano da mettere a mano solo aule e disponibilità.</t>
+          <t xml:space="preserve">  Nel programma il pulsante 'Compila dagli studenti' aggiunge da solo i docenti che compaiono nel foglio</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Aula Lun … Aula Ven: l'aula del docente in ciascun giorno (se è sempre la stessa, si ripete).</t>
+          <t xml:space="preserve">  Studenti e nei gruppi, con i loro strumenti: restano da mettere a mano solo aule e disponibilità.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Viene scritta in testa alla sua colonna nell'orario del giorno.</t>
+          <t xml:space="preserve">  Aula Lun … Aula Ven: l'aula del docente in ciascun giorno (se è sempre la stessa, si ripete).</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Colonne Lun 13:30 … Ven 16:30: scrivi X nelle ore in cui il docente È disponibile. Vuoto = non disponibile.</t>
+          <t xml:space="preserve">  Viene scritta in testa alla sua colonna nell'orario del giorno.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Ore accompagnamento: quante ore a settimana il docente (di pianoforte) fa da pianista accompagnatore. 0 se nessuna.</t>
+          <t xml:space="preserve">  Colonne Lun 13:30 … Ven 16:30: scrivi X nelle ore in cui il docente È disponibile. Vuoto = non disponibile.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Il programma le colloca da solo in coda alle lezioni del docente e nell'orario scrive 'Pianista accomp.'.</t>
+          <t xml:space="preserve">  Ore accompagnamento: quante ore a settimana il docente (di pianoforte) fa da pianista accompagnatore. 0 se nessuna.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Per fissare tu una di queste ore in una fascia precisa, scrivi A al posto della X (solo nelle ultime fasce del giorno).</t>
+          <t xml:space="preserve">  Il programma le colloca da solo in coda alle lezioni del docente e nell'orario scrive 'Pianista accomp.'.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
+          <t xml:space="preserve">  Per fissare tu una di queste ore in una fascia precisa, scrivi A al posto della X (solo nelle ultime fasce del giorno).</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
           <t xml:space="preserve">  Tutte le lezioni del docente (strumento e musica da camera) usano la stessa disponibilità.</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" t="inlineStr"/>
-    </row>
     <row r="26">
-      <c r="A26" s="2" t="inlineStr">
+      <c r="A26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
         <is>
           <t>FOGLIO 'Gruppi LMC' – un rigo per gruppo di musica da camera (classi 3, 4, 5), da 2 a 5 ragazzi.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Scrivi 'Cognome Nome' come nel foglio 'Studenti'. Nel programma c'è il menu a tendina con tutti i ragazzi:</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
+          <t xml:space="preserve">  Scrivi 'Cognome Nome' come nel foglio 'Studenti'. Nel programma c'è il menu a tendina con tutti i ragazzi:</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
           <t xml:space="preserve">  se scrivi solo il cognome e non ci sono omonimi, il nome viene aggiunto da solo.</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" t="inlineStr"/>
-    </row>
     <row r="30">
-      <c r="A30" s="2" t="inlineStr">
+      <c r="A30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
         <is>
           <t>FOGLIO 'Impegni studenti' – le ore in cui un ragazzo NON può venire (sport, catechismo, altro).</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ATTENZIONE: qui è al contrario del foglio Docenti. La X segna l'ora in cui il ragazzo NON c'è.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Chi non ha impegni si lascia con la riga vuota. Nel programma il pulsante 'Compila dagli studenti'</t>
+          <t xml:space="preserve">  ATTENZIONE: qui è al contrario del foglio Docenti. La X segna l'ora in cui il ragazzo NON c'è.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
+          <t xml:space="preserve">  Chi non ha impegni si lascia con la riga vuota. Nel programma il pulsante 'Compila dagli studenti'</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
           <t xml:space="preserve">  ricopia l'elenco dei nomi dal foglio Studenti.</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" t="inlineStr"/>
-    </row>
     <row r="35">
-      <c r="A35" s="2" t="inlineStr">
+      <c r="A35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
         <is>
           <t>FOGLIO 'Abbinamenti fissi' – lezioni già decise, che il programma deve rispettare così come sono.</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Una riga per lezione: docente, studente, tipo (1° strumento, 2° strumento, musica da camera), giorno e ora.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
+          <t xml:space="preserve">  Una riga per lezione: docente, studente, tipo (1° strumento, 2° strumento, musica da camera), giorno e ora.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
           <t xml:space="preserve">  Il tipo si può lasciare vuoto: viene dedotto dal docente. Serve per bloccare gli incastri già concordati.</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" t="inlineStr"/>
-    </row>
     <row r="39">
-      <c r="A39" s="2" t="inlineStr">
-        <is>
-          <t>FOGLIO 'LMI' – laboratori di musica d'insieme (2 ore, orario del MATTINO). Un rigo per laboratorio.</t>
+      <c r="A39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Nella colonna Studente si può scrivere anche il nome di un LABORATORIO del foglio LMI (tipo 'Laboratorio LMI'):</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Il programma NON li calcola: li ricopia così come sono in una pagina dell'orario.</t>
+          <t xml:space="preserve">  in quell'ora vengono occupati il docente e tutti i ragazzi del laboratorio. Il docente si può lasciare vuoto.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Studenti: 'Cognome Nome' separati da virgola. Anche qui il nome viene aggiunto da solo quando non ci sono omonimi.</t>
+          <t xml:space="preserve">  Le 2 ore di 1° strumento non sono per forza attaccate: se le vuoi di seguito, mettile qui in due righe</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" t="inlineStr"/>
+      <c r="A42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  su due ore consecutive (oppure segna '1° strumento attaccato = SI' nel foglio Studenti).</t>
+        </is>
+      </c>
     </row>
     <row r="43">
-      <c r="A43" s="2" t="inlineStr">
-        <is>
-          <t>FOGLIO 'Parametri' – poche regole generali (max rientri, tempo di calcolo). Di norma non serve toccarlo.</t>
-        </is>
-      </c>
+      <c r="A43" t="inlineStr"/>
     </row>
     <row r="44">
-      <c r="A44" t="inlineStr"/>
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>FOGLIO 'LMI' – laboratori di musica d'insieme (2 ore, orario del MATTINO). Un rigo per laboratorio.</t>
+        </is>
+      </c>
     </row>
     <row r="45">
-      <c r="A45" s="2" t="inlineStr">
-        <is>
-          <t>REGOLE FISSE (non modificabili da qui):</t>
+      <c r="A45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Il programma NON li calcola: li ricopia così come sono in una pagina dell'orario. Se però un</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Classi 1 e 2: 2 ore 1° strumento + 1 ora 2° strumento.</t>
+          <t xml:space="preserve">  laboratorio si tiene nel pomeriggio, lo si mette nel foglio 'Abbinamenti fissi' con giorno e ora.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
+          <t xml:space="preserve">  Studenti: 'Cognome Nome' separati da virgola. Anche qui il nome viene aggiunto da solo quando non ci sono omonimi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>FOGLIO 'Parametri' – poche regole generali (max rientri, tempo di calcolo). Di norma non serve toccarlo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>REGOLE FISSE (non modificabili da qui):</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Classi 1 e 2: 2 ore 1° strumento + 1 ora 2° strumento.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
           <t xml:space="preserve">  Classi 3 e 4: 1 ora 1° strumento + 1 ora 2° strumento + 1 ora musica da camera.</t>
         </is>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
+    <row r="54">
+      <c r="A54" t="inlineStr">
         <is>
           <t xml:space="preserve">  Classe 5:     2 ore 1° strumento + 1 ora musica da camera.</t>
         </is>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
+    <row r="55">
+      <c r="A55" t="inlineStr">
         <is>
           <t xml:space="preserve">  Fasce: 13:30-14:30, 14:30-15:30, 15:30-16:30, 16:30-17:30, da lunedì a venerdì.</t>
         </is>
@@ -774,7 +816,7 @@
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="15" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="17" customWidth="1" min="8" max="8"/>
     <col width="13" customWidth="1" min="9" max="9"/>
     <col width="17" customWidth="1" min="10" max="10"/>
     <col width="20" customWidth="1" min="11" max="11"/>
@@ -822,7 +864,7 @@
       </c>
       <c r="H1" s="3" t="inlineStr">
         <is>
-          <t>Ore consecutive (SI/NO)</t>
+          <t>1° strumento attaccato (SI/NO)</t>
         </is>
       </c>
       <c r="I1" s="3" t="inlineStr">
@@ -960,11 +1002,7 @@
           <t>Bianchi</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+      <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr">
         <is>
           <t>NO</t>
@@ -1025,11 +1063,7 @@
           <t>Bianchi</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+      <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr">
         <is>
           <t>NO</t>
@@ -1090,11 +1124,7 @@
           <t>Conti</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+      <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr">
         <is>
           <t>NO</t>
@@ -1155,11 +1185,7 @@
           <t>Marini</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+      <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr">
         <is>
           <t>NO</t>
@@ -1220,11 +1246,7 @@
           <t>Conti</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+      <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr">
         <is>
           <t>NO</t>
@@ -1285,11 +1307,7 @@
           <t>Conti</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+      <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr">
         <is>
           <t>NO</t>
@@ -1350,11 +1368,7 @@
           <t>Bianchi</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+      <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr">
         <is>
           <t>NO</t>
@@ -1484,11 +1498,7 @@
           <t>Bianchi</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+      <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr">
         <is>
           <t>NO</t>
@@ -1549,11 +1559,7 @@
           <t>Bianchi</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+      <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr">
         <is>
           <t>NO</t>
@@ -1679,11 +1685,7 @@
           <t>Verdi</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+      <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr">
         <is>
           <t>NO</t>
@@ -1809,11 +1811,7 @@
           <t>Conti</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+      <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr">
         <is>
           <t>NO</t>
@@ -1874,11 +1872,7 @@
           <t>Bianchi</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+      <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr">
         <is>
           <t>NO</t>
@@ -1939,11 +1933,7 @@
           <t>Lombardi</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+      <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr">
         <is>
           <t>NO</t>
@@ -2004,11 +1994,7 @@
           <t>Marini</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+      <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr">
         <is>
           <t>NO</t>
@@ -2069,11 +2055,7 @@
           <t>Conti</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+      <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr">
         <is>
           <t>SI</t>
@@ -2134,11 +2116,7 @@
           <t>Bianchi</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+      <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr">
         <is>
           <t>SI</t>
@@ -2199,11 +2177,7 @@
           <t>Galli</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+      <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr">
         <is>
           <t>NO</t>
@@ -2264,11 +2238,7 @@
           <t>Conti</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+      <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr">
         <is>
           <t>NO</t>
@@ -2329,11 +2299,7 @@
           <t>Ferrari</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+      <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr">
         <is>
           <t>NO</t>
@@ -2394,11 +2360,7 @@
           <t>Bianchi</t>
         </is>
       </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+      <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr">
         <is>
           <t>NO</t>
@@ -2459,11 +2421,7 @@
           <t>Conti</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+      <c r="H26" t="inlineStr"/>
       <c r="I26" t="inlineStr">
         <is>
           <t>NO</t>
@@ -2520,11 +2478,7 @@
       </c>
       <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr"/>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+      <c r="H27" t="inlineStr"/>
       <c r="I27" t="inlineStr">
         <is>
           <t>NO</t>
@@ -2634,11 +2588,7 @@
       </c>
       <c r="F29" t="inlineStr"/>
       <c r="G29" t="inlineStr"/>
-      <c r="H29" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+      <c r="H29" t="inlineStr"/>
       <c r="I29" t="inlineStr">
         <is>
           <t>NO</t>
@@ -2691,11 +2641,7 @@
       </c>
       <c r="F30" t="inlineStr"/>
       <c r="G30" t="inlineStr"/>
-      <c r="H30" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+      <c r="H30" t="inlineStr"/>
       <c r="I30" t="inlineStr">
         <is>
           <t>NO</t>
@@ -2752,11 +2698,7 @@
       </c>
       <c r="F31" t="inlineStr"/>
       <c r="G31" t="inlineStr"/>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
+      <c r="H31" t="inlineStr"/>
       <c r="I31" t="inlineStr">
         <is>
           <t>NO</t>
@@ -5463,12 +5405,12 @@
   <dimension ref="A1:F1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="44" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -5512,7 +5454,7 @@
       <formula1>=Studenti!$B$2:$B$231</formula1>
     </dataValidation>
     <dataValidation sqref="C2:C202" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"1° strumento,2° strumento,Musica da camera"</formula1>
+      <formula1>"1° strumento,2° strumento,Musica da camera,Laboratorio LMI"</formula1>
     </dataValidation>
     <dataValidation sqref="D2:D202" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Lun,Mar,Mer,Gio,Ven"</formula1>

</xml_diff>